<commit_message>
docs: add use case matrix, Phase 3 prompts, and scenario gaps
Adds RADIANT_Use_Case_Matrix.md defining the v1 imaging scenario
axes (scene type, wavelength regime, target location), locked
design decisions, descriptor schemas, and reference assembly
equations. Adds Phase 3 implementation prompts and reports, the
mixed-train radiometric model doc, scenario testing instructions,
and gaps.md files for scenarios that surfaced issues during
walkthrough review.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scenarios/01_sarah_systems_engineer/1.4_tdi_pushbroom_optimization/outputs/tdi_pushbroom_results.xlsx
+++ b/scenarios/01_sarah_systems_engineer/1.4_tdi_pushbroom_optimization/outputs/tdi_pushbroom_results.xlsx
@@ -538,7 +538,7 @@
         <v>38.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -547,16 +547,16 @@
         <v>0.9959</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.1975</v>
+        <v>0.1155</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0.1</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>5.1</v>
+        <v>4.86</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>0</v>
@@ -581,7 +581,7 @@
         <v>55.3</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -590,16 +590,16 @@
         <v>0.9918</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.1967</v>
+        <v>0.115</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>0.14</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>5.34</v>
+        <v>5.1</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0.24</v>
@@ -624,7 +624,7 @@
         <v>78.59999999999999</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -633,16 +633,16 @@
         <v>0.9836</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.195</v>
+        <v>0.1141</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>0.2</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>5.58</v>
+        <v>5.34</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>0.48</v>
@@ -667,7 +667,7 @@
         <v>111.4</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -676,16 +676,16 @@
         <v>0.9674</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.1918</v>
+        <v>0.1122</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>0.28</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>5.81</v>
+        <v>5.57</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>0.71</v>
@@ -710,7 +710,7 @@
         <v>157.8</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -719,16 +719,16 @@
         <v>0.9355</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.1855</v>
+        <v>0.1085</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>0.4</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>6.05</v>
+        <v>5.81</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>0.95</v>
@@ -753,7 +753,7 @@
         <v>150</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -762,16 +762,16 @@
         <v>0.8735000000000001</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0.1732</v>
+        <v>0.1013</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>0.57</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>6.02</v>
+        <v>5.78</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0.92</v>
@@ -796,7 +796,7 @@
         <v>117.7</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -805,16 +805,16 @@
         <v>0.7568</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.1501</v>
+        <v>0.0878</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0.8</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>5.85</v>
+        <v>5.61</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>0.75</v>
@@ -839,7 +839,7 @@
         <v>100.1</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -848,16 +848,16 @@
         <v>0.6494</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.1288</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0.98</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>5.74</v>
+        <v>5.5</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0.64</v>
@@ -882,7 +882,7 @@
         <v>88.5</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.3115</v>
+        <v>0.1821</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>0.6366000000000001</v>
@@ -891,16 +891,16 @@
         <v>0.5508</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.1092</v>
+        <v>0.0639</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>1.13</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.5656</v>
+        <v>0.479</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>5.66</v>
+        <v>5.42</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>0.5600000000000001</v>

</xml_diff>